<commit_message>
A14: measure 1603-08-08-08-FG bores on the Brennan STEP and stage the row
Brennan's TFA catalog prints the A1/A2 drills as the range 0.44/0.46. The
STEP gives 0.450 for the run and branch bores. Stage the whole row in the
batch-17 table set (Brennan catalog cells + STEP bores, DimSource BRENNAN,
ASSUMED). 1603 now generates 6 of 6 -FG rows with the merged tools; the old
5 are unchanged; vbacheck, dofcheck_tee, allcfg_check and the OCP closed
loop pass. Not shipped, no SolidWorks dry run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QQuceHR8ZUuy6411Z8yX1P
</commit_message>
<xml_diff>
--- a/tools/_out/brennan_yes_20261018/stage/04_DESIGN_TABLES/DesignTable_1603.xlsx
+++ b/tools/_out/brennan_yes_20261018/stage/04_DESIGN_TABLES/DesignTable_1603.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1396,24 +1396,74 @@
           <t>1603-08-08-08-FG</t>
         </is>
       </c>
+      <c r="B13" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.84</v>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>1603-08-08-08-FG</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1/2-14 (A1 (1) NPSM) x 1/2-14 (A1 (2) NPSM) x 1/2-14 (A1 (3) NPSM)</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has the same size only as 1603-08-08-08 (differs by -FG suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-ONLY 2026-10-18] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has the same size only as 1603-08-08-08 (differs by -FG suffix) -&gt; dims NOT copied -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"); D1 / D2 bores measured on BRENNAN_1603-08-08-08-FG.stp 2026-10-20 (A14); sources per cell in CHANGES.csv</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N1, 2701 Y), so 1603-08-08-08 dims are NOT assumed for this SKU; confirm with OMi/Brennan before modelling</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N1, 2701 Y), so 1603-08-08-08 dims are NOT assumed for this SKU; confirm with OMi/Brennan before modelling | 2026-10-18 Brennan = yes (wave2 tee_elbow, staged, not shipped): sizes from the Brennan TFA catalog, end details from the end library; marked $PRP@DimSource BRENNAN (to undo: clear the BRENNAN cells, set the row MISSING, regenerate) | 2026-10-20 A14: D1 / D2 bores 0.450 measured on the Brennan STEP (catalog prints the range 0.44/0.46); the other sizes = the Brennan TFA catalog p.48, all confirmed on the same STEP (nut faces 1.39, stem tips 1.11, nut hex 1.000, body flats 0.875) - staged, not shipped</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1424,6 +1474,11 @@
       <c r="W13" t="inlineStr">
         <is>
           <t>1603-08-08-08-FG</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
         </is>
       </c>
     </row>

</xml_diff>